<commit_message>
Add FBC 13 to Handicaps & Points (Historical)
Points: FBC 13 per-cup points (column P) and cumulative column; Played and
Total/Best/Worst/Average now include FBC 13. Cups: FBC 13 column inserted
before Total with formulas, conditional formatting and filter range moved.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vM3RZF9CPPLM8LSwSGoHo
</commit_message>
<xml_diff>
--- a/Handicaps & Points (Historical).xlsx
+++ b/Handicaps & Points (Historical).xlsx
@@ -18,7 +18,7 @@
     <sheet name="Cups" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Cups!$B$3:$R$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Cups!$B$3:$S$31</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1" calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -3027,7 +3027,11 @@
       <c r="O2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="P2" s="5"/>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>FBC 13</t>
+        </is>
+      </c>
       <c r="Q2" s="5"/>
       <c r="R2" s="19"/>
       <c r="S2" s="8"/>
@@ -3049,8 +3053,7 @@
         <v>Cole</v>
       </c>
       <c r="C3" s="18">
-        <f t="shared" ref="C3:C27" si="0">COUNT(D31:O31)</f>
-        <v>10</v>
+        <f t="shared" ref="C3:C27" si="0">COUNT(D31:P31)</f>
       </c>
       <c r="D3" s="20" t="str">
         <f>IF(COUNT($D31:D31)=0,"X",SUM($D31:D31))</f>
@@ -3100,7 +3103,9 @@
         <f>IF(COUNT($D31:O31)=0,"X",SUM($D31:O31))</f>
         <v>30</v>
       </c>
-      <c r="P3" s="20"/>
+      <c r="P3" s="20">
+        <f>IF(COUNT($D31:P31)=0,"X",SUM($D31:P31))</f>
+      </c>
       <c r="Q3" s="2"/>
       <c r="R3" s="21"/>
       <c r="S3" s="8"/>
@@ -3124,7 +3129,6 @@
       </c>
       <c r="C4" s="18">
         <f t="shared" si="0"/>
-        <v>12</v>
       </c>
       <c r="D4" s="20">
         <f>IF(COUNT($D32:D32)=0,"X",SUM($D32:D32))</f>
@@ -3174,7 +3178,9 @@
         <f>IF(COUNT($D32:O32)=0,"X",SUM($D32:O32))</f>
         <v>50.5</v>
       </c>
-      <c r="P4" s="20"/>
+      <c r="P4" s="20">
+        <f>IF(COUNT($D32:P32)=0,"X",SUM($D32:P32))</f>
+      </c>
       <c r="Q4" s="2"/>
       <c r="R4" s="21"/>
       <c r="S4" s="8"/>
@@ -3197,7 +3203,6 @@
       </c>
       <c r="C5" s="18">
         <f t="shared" si="0"/>
-        <v>2</v>
       </c>
       <c r="D5" s="20" t="str">
         <f>IF(COUNT($D33:D33)=0,"X",SUM($D33:D33))</f>
@@ -3247,7 +3252,9 @@
         <f>IF(COUNT($D33:O33)=0,"X",SUM($D33:O33))</f>
         <v>9</v>
       </c>
-      <c r="P5" s="20"/>
+      <c r="P5" s="20">
+        <f>IF(COUNT($D33:P33)=0,"X",SUM($D33:P33))</f>
+      </c>
       <c r="Q5" s="2"/>
       <c r="R5" s="21"/>
       <c r="S5" s="8"/>
@@ -3271,7 +3278,6 @@
       </c>
       <c r="C6" s="18">
         <f t="shared" si="0"/>
-        <v>10</v>
       </c>
       <c r="D6" s="20" t="str">
         <f>IF(COUNT($D34:D34)=0,"X",SUM($D34:D34))</f>
@@ -3321,7 +3327,9 @@
         <f>IF(COUNT($D34:O34)=0,"X",SUM($D34:O34))</f>
         <v>22</v>
       </c>
-      <c r="P6" s="20"/>
+      <c r="P6" s="20">
+        <f>IF(COUNT($D34:P34)=0,"X",SUM($D34:P34))</f>
+      </c>
       <c r="Q6" s="2"/>
       <c r="R6" s="21"/>
       <c r="S6" s="8"/>
@@ -3344,7 +3352,6 @@
       </c>
       <c r="C7" s="18">
         <f t="shared" si="0"/>
-        <v>6</v>
       </c>
       <c r="D7" s="20" t="str">
         <f>IF(COUNT($D35:D35)=0,"X",SUM($D35:D35))</f>
@@ -3394,7 +3401,9 @@
         <f>IF(COUNT($D35:O35)=0,"X",SUM($D35:O35))</f>
         <v>18.5</v>
       </c>
-      <c r="P7" s="20"/>
+      <c r="P7" s="20">
+        <f>IF(COUNT($D35:P35)=0,"X",SUM($D35:P35))</f>
+      </c>
       <c r="Q7" s="2"/>
       <c r="R7" s="21"/>
       <c r="S7" s="8"/>
@@ -3417,7 +3426,6 @@
       </c>
       <c r="C8" s="18">
         <f t="shared" si="0"/>
-        <v>5</v>
       </c>
       <c r="D8" s="20" t="str">
         <f>IF(COUNT($D36:D36)=0,"X",SUM($D36:D36))</f>
@@ -3467,7 +3475,9 @@
         <f>IF(COUNT($D36:O36)=0,"X",SUM($D36:O36))</f>
         <v>20.5</v>
       </c>
-      <c r="P8" s="20"/>
+      <c r="P8" s="20">
+        <f>IF(COUNT($D36:P36)=0,"X",SUM($D36:P36))</f>
+      </c>
       <c r="Q8" s="2"/>
       <c r="R8" s="21"/>
       <c r="S8" s="8"/>
@@ -3490,7 +3500,6 @@
       </c>
       <c r="C9" s="18">
         <f t="shared" si="0"/>
-        <v>3</v>
       </c>
       <c r="D9" s="20" t="str">
         <f>IF(COUNT($D37:D37)=0,"X",SUM($D37:D37))</f>
@@ -3540,7 +3549,9 @@
         <f>IF(COUNT($D37:O37)=0,"X",SUM($D37:O37))</f>
         <v>7</v>
       </c>
-      <c r="P9" s="20"/>
+      <c r="P9" s="20">
+        <f>IF(COUNT($D37:P37)=0,"X",SUM($D37:P37))</f>
+      </c>
       <c r="Q9" s="2"/>
       <c r="R9" s="21"/>
       <c r="S9" s="8"/>
@@ -3564,7 +3575,6 @@
       </c>
       <c r="C10" s="18">
         <f t="shared" si="0"/>
-        <v>12</v>
       </c>
       <c r="D10" s="20">
         <f>IF(COUNT($D38:D38)=0,"X",SUM($D38:D38))</f>
@@ -3614,7 +3624,9 @@
         <f>IF(COUNT($D38:O38)=0,"X",SUM($D38:O38))</f>
         <v>46</v>
       </c>
-      <c r="P10" s="20"/>
+      <c r="P10" s="20">
+        <f>IF(COUNT($D38:P38)=0,"X",SUM($D38:P38))</f>
+      </c>
       <c r="Q10" s="2"/>
       <c r="R10" s="21"/>
       <c r="S10" s="8"/>
@@ -3638,7 +3650,6 @@
       </c>
       <c r="C11" s="18">
         <f t="shared" si="0"/>
-        <v>12</v>
       </c>
       <c r="D11" s="20">
         <f>IF(COUNT($D39:D39)=0,"X",SUM($D39:D39))</f>
@@ -3688,7 +3699,9 @@
         <f>IF(COUNT($D39:O39)=0,"X",SUM($D39:O39))</f>
         <v>36.5</v>
       </c>
-      <c r="P11" s="20"/>
+      <c r="P11" s="20">
+        <f>IF(COUNT($D39:P39)=0,"X",SUM($D39:P39))</f>
+      </c>
       <c r="Q11" s="2"/>
       <c r="R11" s="21"/>
       <c r="S11" s="8"/>
@@ -3712,7 +3725,6 @@
       </c>
       <c r="C12" s="18">
         <f t="shared" si="0"/>
-        <v>11</v>
       </c>
       <c r="D12" s="20" t="str">
         <f>IF(COUNT($D40:D40)=0,"X",SUM($D40:D40))</f>
@@ -3762,7 +3774,9 @@
         <f>IF(COUNT($D40:O40)=0,"X",SUM($D40:O40))</f>
         <v>30</v>
       </c>
-      <c r="P12" s="20"/>
+      <c r="P12" s="20">
+        <f>IF(COUNT($D40:P40)=0,"X",SUM($D40:P40))</f>
+      </c>
       <c r="Q12" s="2"/>
       <c r="R12" s="21"/>
       <c r="S12" s="8"/>
@@ -3786,7 +3800,6 @@
       </c>
       <c r="C13" s="18">
         <f t="shared" si="0"/>
-        <v>11</v>
       </c>
       <c r="D13" s="20" t="str">
         <f>IF(COUNT($D41:D41)=0,"X",SUM($D41:D41))</f>
@@ -3836,7 +3849,9 @@
         <f>IF(COUNT($D41:O41)=0,"X",SUM($D41:O41))</f>
         <v>42</v>
       </c>
-      <c r="P13" s="20"/>
+      <c r="P13" s="20">
+        <f>IF(COUNT($D41:P41)=0,"X",SUM($D41:P41))</f>
+      </c>
       <c r="Q13" s="2"/>
       <c r="R13" s="21"/>
       <c r="S13" s="8"/>
@@ -3860,7 +3875,6 @@
       </c>
       <c r="C14" s="18">
         <f t="shared" si="0"/>
-        <v>7</v>
       </c>
       <c r="D14" s="20" t="str">
         <f>IF(COUNT($D42:D42)=0,"X",SUM($D42:D42))</f>
@@ -3910,7 +3924,9 @@
         <f>IF(COUNT($D42:O42)=0,"X",SUM($D42:O42))</f>
         <v>31</v>
       </c>
-      <c r="P14" s="20"/>
+      <c r="P14" s="20">
+        <f>IF(COUNT($D42:P42)=0,"X",SUM($D42:P42))</f>
+      </c>
       <c r="Q14" s="2"/>
       <c r="R14" s="21"/>
       <c r="S14" s="8"/>
@@ -3934,7 +3950,6 @@
       </c>
       <c r="C15" s="18">
         <f t="shared" si="0"/>
-        <v>12</v>
       </c>
       <c r="D15" s="20">
         <f>IF(COUNT($D43:D43)=0,"X",SUM($D43:D43))</f>
@@ -3984,7 +3999,9 @@
         <f>IF(COUNT($D43:O43)=0,"X",SUM($D43:O43))</f>
         <v>43</v>
       </c>
-      <c r="P15" s="20"/>
+      <c r="P15" s="20">
+        <f>IF(COUNT($D43:P43)=0,"X",SUM($D43:P43))</f>
+      </c>
       <c r="Q15" s="2"/>
       <c r="R15" s="21"/>
       <c r="S15" s="8"/>
@@ -4008,7 +4025,6 @@
       </c>
       <c r="C16" s="18">
         <f t="shared" si="0"/>
-        <v>11</v>
       </c>
       <c r="D16" s="20">
         <f>IF(COUNT($D44:D44)=0,"X",SUM($D44:D44))</f>
@@ -4058,7 +4074,9 @@
         <f>IF(COUNT($D44:O44)=0,"X",SUM($D44:O44))</f>
         <v>37</v>
       </c>
-      <c r="P16" s="20"/>
+      <c r="P16" s="20">
+        <f>IF(COUNT($D44:P44)=0,"X",SUM($D44:P44))</f>
+      </c>
       <c r="Q16" s="2"/>
       <c r="R16" s="21"/>
       <c r="S16" s="8"/>
@@ -4082,7 +4100,6 @@
       </c>
       <c r="C17" s="18">
         <f t="shared" si="0"/>
-        <v>12</v>
       </c>
       <c r="D17" s="20">
         <f>IF(COUNT($D45:D45)=0,"X",SUM($D45:D45))</f>
@@ -4132,7 +4149,9 @@
         <f>IF(COUNT($D45:O45)=0,"X",SUM($D45:O45))</f>
         <v>46</v>
       </c>
-      <c r="P17" s="20"/>
+      <c r="P17" s="20">
+        <f>IF(COUNT($D45:P45)=0,"X",SUM($D45:P45))</f>
+      </c>
       <c r="Q17" s="2"/>
       <c r="R17" s="21"/>
       <c r="S17" s="8"/>
@@ -4156,7 +4175,6 @@
       </c>
       <c r="C18" s="18">
         <f t="shared" si="0"/>
-        <v>12</v>
       </c>
       <c r="D18" s="20">
         <f>IF(COUNT($D46:D46)=0,"X",SUM($D46:D46))</f>
@@ -4206,7 +4224,9 @@
         <f>IF(COUNT($D46:O46)=0,"X",SUM($D46:O46))</f>
         <v>41</v>
       </c>
-      <c r="P18" s="20"/>
+      <c r="P18" s="20">
+        <f>IF(COUNT($D46:P46)=0,"X",SUM($D46:P46))</f>
+      </c>
       <c r="Q18" s="2"/>
       <c r="R18" s="21"/>
       <c r="S18" s="8"/>
@@ -4230,7 +4250,6 @@
       </c>
       <c r="C19" s="18">
         <f t="shared" si="0"/>
-        <v>11</v>
       </c>
       <c r="D19" s="20">
         <f>IF(COUNT($D47:D47)=0,"X",SUM($D47:D47))</f>
@@ -4280,7 +4299,9 @@
         <f>IF(COUNT($D47:O47)=0,"X",SUM($D47:O47))</f>
         <v>28.5</v>
       </c>
-      <c r="P19" s="20"/>
+      <c r="P19" s="20">
+        <f>IF(COUNT($D47:P47)=0,"X",SUM($D47:P47))</f>
+      </c>
       <c r="Q19" s="2"/>
       <c r="R19" s="21"/>
       <c r="S19" s="8"/>
@@ -4304,7 +4325,6 @@
       </c>
       <c r="C20" s="18">
         <f t="shared" si="0"/>
-        <v>8</v>
       </c>
       <c r="D20" s="20" t="str">
         <f>IF(COUNT($D48:D48)=0,"X",SUM($D48:D48))</f>
@@ -4354,7 +4374,9 @@
         <f>IF(COUNT($D48:O48)=0,"X",SUM($D48:O48))</f>
         <v>28</v>
       </c>
-      <c r="P20" s="20"/>
+      <c r="P20" s="20">
+        <f>IF(COUNT($D48:P48)=0,"X",SUM($D48:P48))</f>
+      </c>
       <c r="Q20" s="2"/>
       <c r="R20" s="21"/>
       <c r="S20" s="8"/>
@@ -4378,7 +4400,6 @@
       </c>
       <c r="C21" s="18">
         <f t="shared" si="0"/>
-        <v>6</v>
       </c>
       <c r="D21" s="20" t="str">
         <f>IF(COUNT($D49:D49)=0,"X",SUM($D49:D49))</f>
@@ -4428,7 +4449,9 @@
         <f>IF(COUNT($D49:O49)=0,"X",SUM($D49:O49))</f>
         <v>21</v>
       </c>
-      <c r="P21" s="20"/>
+      <c r="P21" s="20">
+        <f>IF(COUNT($D49:P49)=0,"X",SUM($D49:P49))</f>
+      </c>
       <c r="Q21" s="2"/>
       <c r="R21" s="21"/>
       <c r="S21" s="8"/>
@@ -4451,7 +4474,6 @@
       </c>
       <c r="C22" s="18">
         <f t="shared" si="0"/>
-        <v>4</v>
       </c>
       <c r="D22" s="20" t="str">
         <f>IF(COUNT($D50:D50)=0,"X",SUM($D50:D50))</f>
@@ -4501,7 +4523,9 @@
         <f>IF(COUNT($D50:O50)=0,"X",SUM($D50:O50))</f>
         <v>18.5</v>
       </c>
-      <c r="P22" s="20"/>
+      <c r="P22" s="20">
+        <f>IF(COUNT($D50:P50)=0,"X",SUM($D50:P50))</f>
+      </c>
       <c r="Q22" s="2"/>
       <c r="R22" s="21"/>
       <c r="S22" s="8"/>
@@ -4524,7 +4548,6 @@
       </c>
       <c r="C23" s="18">
         <f t="shared" si="0"/>
-        <v>2</v>
       </c>
       <c r="D23" s="20" t="str">
         <f>IF(COUNT($D51:D51)=0,"X",SUM($D51:D51))</f>
@@ -4574,7 +4597,9 @@
         <f>IF(COUNT($D51:O51)=0,"X",SUM($D51:O51))</f>
         <v>2.5</v>
       </c>
-      <c r="P23" s="20"/>
+      <c r="P23" s="20">
+        <f>IF(COUNT($D51:P51)=0,"X",SUM($D51:P51))</f>
+      </c>
       <c r="Q23" s="2"/>
       <c r="R23" s="21"/>
       <c r="S23" s="8"/>
@@ -4598,7 +4623,6 @@
       </c>
       <c r="C24" s="18">
         <f t="shared" si="0"/>
-        <v>7</v>
       </c>
       <c r="D24" s="20">
         <f>IF(COUNT($D52:D52)=0,"X",SUM($D52:D52))</f>
@@ -4648,7 +4672,9 @@
         <f>IF(COUNT($D52:O52)=0,"X",SUM($D52:O52))</f>
         <v>27</v>
       </c>
-      <c r="P24" s="20"/>
+      <c r="P24" s="20">
+        <f>IF(COUNT($D52:P52)=0,"X",SUM($D52:P52))</f>
+      </c>
       <c r="Q24" s="2"/>
       <c r="R24" s="21"/>
       <c r="S24" s="8"/>
@@ -4672,7 +4698,6 @@
       </c>
       <c r="C25" s="18">
         <f t="shared" si="0"/>
-        <v>11</v>
       </c>
       <c r="D25" s="20">
         <f>IF(COUNT($D53:D53)=0,"X",SUM($D53:D53))</f>
@@ -4722,7 +4747,9 @@
         <f>IF(COUNT($D53:O53)=0,"X",SUM($D53:O53))</f>
         <v>27</v>
       </c>
-      <c r="P25" s="20"/>
+      <c r="P25" s="20">
+        <f>IF(COUNT($D53:P53)=0,"X",SUM($D53:P53))</f>
+      </c>
       <c r="Q25" s="2"/>
       <c r="R25" s="21"/>
       <c r="S25" s="8"/>
@@ -4746,7 +4773,6 @@
       </c>
       <c r="C26" s="18">
         <f t="shared" si="0"/>
-        <v>8</v>
       </c>
       <c r="D26" s="20" t="str">
         <f>IF(COUNT($D54:D54)=0,"X",SUM($D54:D54))</f>
@@ -4796,7 +4822,9 @@
         <f>IF(COUNT($D54:O54)=0,"X",SUM($D54:O54))</f>
         <v>28.5</v>
       </c>
-      <c r="P26" s="20"/>
+      <c r="P26" s="20">
+        <f>IF(COUNT($D54:P54)=0,"X",SUM($D54:P54))</f>
+      </c>
       <c r="Q26" s="2"/>
       <c r="R26" s="21"/>
       <c r="S26" s="8"/>
@@ -4820,7 +4848,6 @@
       </c>
       <c r="C27" s="18">
         <f t="shared" si="0"/>
-        <v>10</v>
       </c>
       <c r="D27" s="20" t="str">
         <f>IF(COUNT($D55:D55)=0,"X",SUM($D55:D55))</f>
@@ -4870,7 +4897,9 @@
         <f>IF(COUNT($D55:O55)=0,"X",SUM($D55:O55))</f>
         <v>32.5</v>
       </c>
-      <c r="P27" s="20"/>
+      <c r="P27" s="20">
+        <f>IF(COUNT($D55:P55)=0,"X",SUM($D55:P55))</f>
+      </c>
       <c r="Q27" s="2"/>
       <c r="R27" s="21"/>
       <c r="S27" s="8"/>
@@ -4973,7 +5002,10 @@
       <c r="O29" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="P29" s="19"/>
+      <c r="P29" s="19" t="str">
+        <f>P2</f>
+        <v>FBC 13</v>
+      </c>
       <c r="Q29" s="17" t="s">
         <v>48</v>
       </c>
@@ -5038,7 +5070,11 @@
       <c r="O30" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="P30" s="19"/>
+      <c r="P30" s="19" t="inlineStr">
+        <is>
+          <t>Frisco</t>
+        </is>
+      </c>
       <c r="Q30" s="17"/>
       <c r="R30" s="19"/>
       <c r="S30" s="19"/>
@@ -5096,22 +5132,20 @@
       <c r="O31" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="P31" s="20"/>
+      <c r="P31" s="20">
+        <v>4</v>
+      </c>
       <c r="Q31" s="20">
-        <f t="shared" ref="Q31:Q55" si="2">SUM(D31:O31)</f>
-        <v>30</v>
+        <f t="shared" ref="Q31:Q55" si="2">SUM(D31:P31)</f>
       </c>
       <c r="R31" s="20">
-        <f t="shared" ref="R31:R55" si="3">MAX(D31:O31)</f>
-        <v>4.5</v>
+        <f t="shared" ref="R31:R55" si="3">MAX(D31:P31)</f>
       </c>
       <c r="S31" s="20">
-        <f t="shared" ref="S31:S55" si="4">MIN(D31:O31)</f>
-        <v>0.5</v>
+        <f t="shared" ref="S31:S55" si="4">MIN(D31:P31)</f>
       </c>
       <c r="T31" s="21">
-        <f t="shared" ref="T31:T55" si="5">AVERAGE(D31:O31)</f>
-        <v>3</v>
+        <f t="shared" ref="T31:T55" si="5">AVERAGE(D31:P31)</f>
       </c>
       <c r="U31" s="20">
         <f t="shared" ref="U31:U55" si="6">R31-S31</f>
@@ -5169,22 +5203,20 @@
       <c r="O32" s="20">
         <v>6.5</v>
       </c>
-      <c r="P32" s="20"/>
+      <c r="P32" s="20">
+        <v>2</v>
+      </c>
       <c r="Q32" s="20">
         <f t="shared" si="2"/>
-        <v>50.5</v>
       </c>
       <c r="R32" s="20">
         <f t="shared" si="3"/>
-        <v>6.5</v>
       </c>
       <c r="S32" s="20">
         <f t="shared" si="4"/>
-        <v>2</v>
       </c>
       <c r="T32" s="21">
         <f t="shared" si="5"/>
-        <v>4.208333333333333</v>
       </c>
       <c r="U32" s="20">
         <f t="shared" si="6"/>
@@ -5237,22 +5269,20 @@
       <c r="O33" s="20">
         <v>6</v>
       </c>
-      <c r="P33" s="20"/>
+      <c r="P33" s="20">
+        <v>1.5</v>
+      </c>
       <c r="Q33" s="20">
         <f t="shared" si="2"/>
-        <v>9</v>
       </c>
       <c r="R33" s="20">
         <f t="shared" si="3"/>
-        <v>6</v>
       </c>
       <c r="S33" s="20">
         <f t="shared" si="4"/>
-        <v>3</v>
       </c>
       <c r="T33" s="21">
         <f t="shared" si="5"/>
-        <v>4.5</v>
       </c>
       <c r="U33" s="20">
         <f t="shared" si="6"/>
@@ -5306,22 +5336,22 @@
       <c r="O34" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="P34" s="20"/>
+      <c r="P34" s="20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="Q34" s="20">
         <f t="shared" si="2"/>
-        <v>22</v>
       </c>
       <c r="R34" s="20">
         <f t="shared" si="3"/>
-        <v>3.5</v>
       </c>
       <c r="S34" s="20">
         <f t="shared" si="4"/>
-        <v>1</v>
       </c>
       <c r="T34" s="21">
         <f t="shared" si="5"/>
-        <v>2.2</v>
       </c>
       <c r="U34" s="20">
         <f t="shared" si="6"/>
@@ -5374,22 +5404,20 @@
       <c r="O35" s="20">
         <v>4</v>
       </c>
-      <c r="P35" s="20"/>
+      <c r="P35" s="20">
+        <v>4</v>
+      </c>
       <c r="Q35" s="20">
         <f t="shared" si="2"/>
-        <v>18.5</v>
       </c>
       <c r="R35" s="20">
         <f t="shared" si="3"/>
-        <v>4</v>
       </c>
       <c r="S35" s="20">
         <f t="shared" si="4"/>
-        <v>2</v>
       </c>
       <c r="T35" s="21">
         <f t="shared" si="5"/>
-        <v>3.0833333333333335</v>
       </c>
       <c r="U35" s="20">
         <f t="shared" si="6"/>
@@ -5442,22 +5470,20 @@
       <c r="O36" s="20">
         <v>5</v>
       </c>
-      <c r="P36" s="20"/>
+      <c r="P36" s="20">
+        <v>4</v>
+      </c>
       <c r="Q36" s="20">
         <f t="shared" si="2"/>
-        <v>20.5</v>
       </c>
       <c r="R36" s="20">
         <f t="shared" si="3"/>
-        <v>5</v>
       </c>
       <c r="S36" s="20">
         <f t="shared" si="4"/>
-        <v>1.5</v>
       </c>
       <c r="T36" s="21">
         <f t="shared" si="5"/>
-        <v>4.1</v>
       </c>
       <c r="U36" s="20">
         <f t="shared" si="6"/>
@@ -5510,22 +5536,20 @@
       <c r="O37" s="20">
         <v>1</v>
       </c>
-      <c r="P37" s="20"/>
+      <c r="P37" s="20">
+        <v>2.5</v>
+      </c>
       <c r="Q37" s="20">
         <f t="shared" si="2"/>
-        <v>7</v>
       </c>
       <c r="R37" s="20">
         <f t="shared" si="3"/>
-        <v>3</v>
       </c>
       <c r="S37" s="20">
         <f t="shared" si="4"/>
-        <v>1</v>
       </c>
       <c r="T37" s="21">
         <f t="shared" si="5"/>
-        <v>2.3333333333333335</v>
       </c>
       <c r="U37" s="20">
         <f t="shared" si="6"/>
@@ -5579,22 +5603,20 @@
       <c r="O38" s="20">
         <v>3.5</v>
       </c>
-      <c r="P38" s="20"/>
+      <c r="P38" s="20">
+        <v>4.5</v>
+      </c>
       <c r="Q38" s="20">
         <f t="shared" si="2"/>
-        <v>46</v>
       </c>
       <c r="R38" s="20">
         <f t="shared" si="3"/>
-        <v>5.5</v>
       </c>
       <c r="S38" s="20">
         <f t="shared" si="4"/>
-        <v>2.5</v>
       </c>
       <c r="T38" s="21">
         <f t="shared" si="5"/>
-        <v>3.8333333333333335</v>
       </c>
       <c r="U38" s="20">
         <f t="shared" si="6"/>
@@ -5648,22 +5670,20 @@
       <c r="O39" s="20">
         <v>6.5</v>
       </c>
-      <c r="P39" s="20"/>
+      <c r="P39" s="20">
+        <v>5</v>
+      </c>
       <c r="Q39" s="20">
         <f t="shared" si="2"/>
-        <v>36.5</v>
       </c>
       <c r="R39" s="20">
         <f t="shared" si="3"/>
-        <v>6.5</v>
       </c>
       <c r="S39" s="20">
         <f t="shared" si="4"/>
-        <v>0.5</v>
       </c>
       <c r="T39" s="21">
         <f t="shared" si="5"/>
-        <v>3.0416666666666665</v>
       </c>
       <c r="U39" s="20">
         <f t="shared" si="6"/>
@@ -5717,22 +5737,20 @@
       <c r="O40" s="20">
         <v>4</v>
       </c>
-      <c r="P40" s="20"/>
+      <c r="P40" s="20">
+        <v>3</v>
+      </c>
       <c r="Q40" s="20">
         <f t="shared" si="2"/>
-        <v>30</v>
       </c>
       <c r="R40" s="20">
         <f t="shared" si="3"/>
-        <v>4.5</v>
       </c>
       <c r="S40" s="20">
         <f t="shared" si="4"/>
-        <v>0.5</v>
       </c>
       <c r="T40" s="21">
         <f t="shared" si="5"/>
-        <v>2.727272727272727</v>
       </c>
       <c r="U40" s="20">
         <f t="shared" si="6"/>
@@ -5786,22 +5804,20 @@
       <c r="O41" s="20">
         <v>4</v>
       </c>
-      <c r="P41" s="20"/>
+      <c r="P41" s="20">
+        <v>4.5</v>
+      </c>
       <c r="Q41" s="20">
         <f t="shared" si="2"/>
-        <v>42</v>
       </c>
       <c r="R41" s="20">
         <f t="shared" si="3"/>
-        <v>5.5</v>
       </c>
       <c r="S41" s="20">
         <f t="shared" si="4"/>
-        <v>0</v>
       </c>
       <c r="T41" s="21">
         <f t="shared" si="5"/>
-        <v>3.8181818181818183</v>
       </c>
       <c r="U41" s="20">
         <f t="shared" si="6"/>
@@ -5875,22 +5891,20 @@
       <c r="O42" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="P42" s="20"/>
+      <c r="P42" s="20">
+        <v>3.5</v>
+      </c>
       <c r="Q42" s="20">
         <f t="shared" si="2"/>
-        <v>31</v>
       </c>
       <c r="R42" s="20">
         <f t="shared" si="3"/>
-        <v>7</v>
       </c>
       <c r="S42" s="20">
         <f t="shared" si="4"/>
-        <v>2.5</v>
       </c>
       <c r="T42" s="21">
         <f t="shared" si="5"/>
-        <v>4.428571428571429</v>
       </c>
       <c r="U42" s="20">
         <f t="shared" si="6"/>
@@ -5964,22 +5978,20 @@
       <c r="O43" s="20">
         <v>4</v>
       </c>
-      <c r="P43" s="20"/>
+      <c r="P43" s="20">
+        <v>3.5</v>
+      </c>
       <c r="Q43" s="20">
         <f t="shared" si="2"/>
-        <v>43</v>
       </c>
       <c r="R43" s="20">
         <f t="shared" si="3"/>
-        <v>6.5</v>
       </c>
       <c r="S43" s="20">
         <f t="shared" si="4"/>
-        <v>0.5</v>
       </c>
       <c r="T43" s="21">
         <f t="shared" si="5"/>
-        <v>3.5833333333333335</v>
       </c>
       <c r="U43" s="20">
         <f t="shared" si="6"/>
@@ -6053,22 +6065,20 @@
       <c r="O44" s="20">
         <v>4.5</v>
       </c>
-      <c r="P44" s="20"/>
+      <c r="P44" s="20">
+        <v>3.5</v>
+      </c>
       <c r="Q44" s="20">
         <f t="shared" si="2"/>
-        <v>37</v>
       </c>
       <c r="R44" s="20">
         <f t="shared" si="3"/>
-        <v>5.5</v>
       </c>
       <c r="S44" s="20">
         <f t="shared" si="4"/>
-        <v>2</v>
       </c>
       <c r="T44" s="21">
         <f t="shared" si="5"/>
-        <v>3.3636363636363638</v>
       </c>
       <c r="U44" s="20">
         <f t="shared" si="6"/>
@@ -6142,22 +6152,20 @@
       <c r="O45" s="20">
         <v>3.5</v>
       </c>
-      <c r="P45" s="20"/>
+      <c r="P45" s="20">
+        <v>5</v>
+      </c>
       <c r="Q45" s="20">
         <f t="shared" si="2"/>
-        <v>46</v>
       </c>
       <c r="R45" s="20">
         <f t="shared" si="3"/>
-        <v>6.5</v>
       </c>
       <c r="S45" s="20">
         <f t="shared" si="4"/>
-        <v>1</v>
       </c>
       <c r="T45" s="21">
         <f t="shared" si="5"/>
-        <v>3.8333333333333335</v>
       </c>
       <c r="U45" s="20">
         <f t="shared" si="6"/>
@@ -6231,22 +6239,20 @@
       <c r="O46" s="20">
         <v>3</v>
       </c>
-      <c r="P46" s="20"/>
+      <c r="P46" s="20">
+        <v>1.5</v>
+      </c>
       <c r="Q46" s="20">
         <f t="shared" si="2"/>
-        <v>41</v>
       </c>
       <c r="R46" s="20">
         <f t="shared" si="3"/>
-        <v>5.5</v>
       </c>
       <c r="S46" s="20">
         <f t="shared" si="4"/>
-        <v>1.5</v>
       </c>
       <c r="T46" s="21">
         <f t="shared" si="5"/>
-        <v>3.4166666666666665</v>
       </c>
       <c r="U46" s="20">
         <f t="shared" si="6"/>
@@ -6319,22 +6325,20 @@
       <c r="O47" s="20">
         <v>5.5</v>
       </c>
-      <c r="P47" s="20"/>
+      <c r="P47" s="20">
+        <v>1.5</v>
+      </c>
       <c r="Q47" s="20">
         <f t="shared" si="2"/>
-        <v>28.5</v>
       </c>
       <c r="R47" s="20">
         <f t="shared" si="3"/>
-        <v>5.5</v>
       </c>
       <c r="S47" s="20">
         <f t="shared" si="4"/>
-        <v>0</v>
       </c>
       <c r="T47" s="21">
         <f t="shared" si="5"/>
-        <v>2.590909090909091</v>
       </c>
       <c r="U47" s="20">
         <f t="shared" si="6"/>
@@ -6407,22 +6411,20 @@
       <c r="O48" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="P48" s="20"/>
+      <c r="P48" s="20">
+        <v>2</v>
+      </c>
       <c r="Q48" s="20">
         <f t="shared" si="2"/>
-        <v>28</v>
       </c>
       <c r="R48" s="20">
         <f t="shared" si="3"/>
-        <v>5.5</v>
       </c>
       <c r="S48" s="20">
         <f t="shared" si="4"/>
-        <v>2.5</v>
       </c>
       <c r="T48" s="21">
         <f t="shared" si="5"/>
-        <v>3.5</v>
       </c>
       <c r="U48" s="20">
         <f t="shared" si="6"/>
@@ -6495,22 +6497,20 @@
       <c r="O49" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="P49" s="20"/>
+      <c r="P49" s="20">
+        <v>5.5</v>
+      </c>
       <c r="Q49" s="20">
         <f t="shared" si="2"/>
-        <v>21</v>
       </c>
       <c r="R49" s="20">
         <f t="shared" si="3"/>
-        <v>5.5</v>
       </c>
       <c r="S49" s="20">
         <f t="shared" si="4"/>
-        <v>2</v>
       </c>
       <c r="T49" s="21">
         <f t="shared" si="5"/>
-        <v>3.5</v>
       </c>
       <c r="U49" s="20">
         <f t="shared" si="6"/>
@@ -6582,22 +6582,20 @@
       <c r="O50" s="20">
         <v>5</v>
       </c>
-      <c r="P50" s="20"/>
+      <c r="P50" s="20">
+        <v>2.5</v>
+      </c>
       <c r="Q50" s="20">
         <f t="shared" si="2"/>
-        <v>18.5</v>
       </c>
       <c r="R50" s="20">
         <f t="shared" si="3"/>
-        <v>6</v>
       </c>
       <c r="S50" s="20">
         <f t="shared" si="4"/>
-        <v>2</v>
       </c>
       <c r="T50" s="21">
         <f t="shared" si="5"/>
-        <v>4.625</v>
       </c>
       <c r="U50" s="20">
         <f t="shared" si="6"/>
@@ -6669,22 +6667,20 @@
       <c r="O51" s="20">
         <v>1</v>
       </c>
-      <c r="P51" s="20"/>
+      <c r="P51" s="20">
+        <v>4.5</v>
+      </c>
       <c r="Q51" s="20">
         <f t="shared" si="2"/>
-        <v>2.5</v>
       </c>
       <c r="R51" s="20">
         <f t="shared" si="3"/>
-        <v>1.5</v>
       </c>
       <c r="S51" s="20">
         <f t="shared" si="4"/>
-        <v>1</v>
       </c>
       <c r="T51" s="21">
         <f t="shared" si="5"/>
-        <v>1.25</v>
       </c>
       <c r="U51" s="20">
         <f t="shared" si="6"/>
@@ -6757,22 +6753,20 @@
       <c r="O52" s="20">
         <v>6</v>
       </c>
-      <c r="P52" s="20"/>
+      <c r="P52" s="20">
+        <v>2.5</v>
+      </c>
       <c r="Q52" s="20">
         <f t="shared" si="2"/>
-        <v>27</v>
       </c>
       <c r="R52" s="20">
         <f t="shared" si="3"/>
-        <v>6</v>
       </c>
       <c r="S52" s="20">
         <f t="shared" si="4"/>
-        <v>0</v>
       </c>
       <c r="T52" s="21">
         <f t="shared" si="5"/>
-        <v>3.857142857142857</v>
       </c>
       <c r="U52" s="20">
         <f t="shared" si="6"/>
@@ -6845,22 +6839,20 @@
       <c r="O53" s="20">
         <v>1.5</v>
       </c>
-      <c r="P53" s="20"/>
+      <c r="P53" s="20">
+        <v>2</v>
+      </c>
       <c r="Q53" s="20">
         <f t="shared" si="2"/>
-        <v>27</v>
       </c>
       <c r="R53" s="20">
         <f t="shared" si="3"/>
-        <v>5.5</v>
       </c>
       <c r="S53" s="20">
         <f t="shared" si="4"/>
-        <v>0.5</v>
       </c>
       <c r="T53" s="21">
         <f t="shared" si="5"/>
-        <v>2.4545454545454546</v>
       </c>
       <c r="U53" s="20">
         <f t="shared" si="6"/>
@@ -6933,22 +6925,20 @@
       <c r="O54" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="P54" s="20"/>
+      <c r="P54" s="20">
+        <v>4.5</v>
+      </c>
       <c r="Q54" s="20">
         <f t="shared" si="2"/>
-        <v>28.5</v>
       </c>
       <c r="R54" s="20">
         <f t="shared" si="3"/>
-        <v>5.5</v>
       </c>
       <c r="S54" s="20">
         <f t="shared" si="4"/>
-        <v>2</v>
       </c>
       <c r="T54" s="21">
         <f t="shared" si="5"/>
-        <v>3.5625</v>
       </c>
       <c r="U54" s="20">
         <f t="shared" si="6"/>
@@ -7021,22 +7011,20 @@
       <c r="O55" s="20">
         <v>1.5</v>
       </c>
-      <c r="P55" s="20"/>
+      <c r="P55" s="20">
+        <v>1</v>
+      </c>
       <c r="Q55" s="20">
         <f t="shared" si="2"/>
-        <v>32.5</v>
       </c>
       <c r="R55" s="20">
         <f t="shared" si="3"/>
-        <v>6</v>
       </c>
       <c r="S55" s="20">
         <f t="shared" si="4"/>
-        <v>1</v>
       </c>
       <c r="T55" s="21">
         <f t="shared" si="5"/>
-        <v>3.25</v>
       </c>
       <c r="U55" s="20">
         <f t="shared" si="6"/>
@@ -7490,7 +7478,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:U40"/>
+  <dimension ref="A1:V40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="10.33203125" customWidth="1"/>
@@ -7502,11 +7490,11 @@
     <col min="9" max="9" width="7.1640625" customWidth="1"/>
     <col min="10" max="11" width="7.5" customWidth="1"/>
     <col min="12" max="13" width="7.33203125" customWidth="1"/>
-    <col min="14" max="14" width="8" customWidth="1"/>
-    <col min="17" max="18" width="10" customWidth="1"/>
+    <col min="14" max="15" width="8" customWidth="1"/>
+    <col min="18" max="19" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7528,8 +7516,9 @@
       <c r="S1" s="2"/>
       <c r="T1" s="2"/>
       <c r="U1" s="2"/>
-    </row>
-    <row r="2" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V1" s="2"/>
+    </row>
+    <row r="2" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
       <c r="B2" s="15" t="str">
         <f>Handicaps!B2</f>
@@ -7571,23 +7560,28 @@
       <c r="N2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="O2" s="7" t="inlineStr">
+        <is>
+          <t>FBC 13</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="P2" s="7" t="s">
+      <c r="Q2" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="Q2" s="7" t="s">
+      <c r="R2" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="R2" s="7" t="s">
+      <c r="S2" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="S2" s="2"/>
       <c r="T2" s="2"/>
       <c r="U2" s="2"/>
-    </row>
-    <row r="3" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V2" s="2"/>
+    </row>
+    <row r="3" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="2" t="s">
         <v>32</v>
@@ -7629,26 +7623,25 @@
         <v>1</v>
       </c>
       <c r="O3" s="24">
-        <f t="shared" ref="O3:O4" si="0">SUM(C3:N3)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P3" s="24">
+        <f t="shared" ref="P3:P4" si="0">SUM(C3:O3)</f>
+      </c>
+      <c r="Q3" s="24">
         <f>VLOOKUP($B3,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>12</v>
-      </c>
-      <c r="Q3" s="25">
-        <f t="shared" ref="Q3:Q4" si="1">O3/P3</f>
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="R3" s="24">
-        <f t="shared" ref="R3:R4" si="2">P3-O3</f>
-        <v>2</v>
-      </c>
-      <c r="S3" s="2"/>
+      </c>
+      <c r="R3" s="25">
+        <f t="shared" ref="R3:R4" si="1">P3/Q3</f>
+      </c>
+      <c r="S3" s="24">
+        <f t="shared" ref="S3:S4" si="2">Q3-P3</f>
+      </c>
       <c r="T3" s="2"/>
       <c r="U3" s="2"/>
-    </row>
-    <row r="4" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V3" s="2"/>
+    </row>
+    <row r="4" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="2" t="s">
         <v>71</v>
@@ -7690,26 +7683,25 @@
         <v>0</v>
       </c>
       <c r="O4" s="24">
+        <v>1</v>
+      </c>
+      <c r="P4" s="24">
         <f t="shared" si="0"/>
-        <v>9</v>
-      </c>
-      <c r="P4" s="24">
+      </c>
+      <c r="Q4" s="24">
         <f>VLOOKUP($B4,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>12</v>
-      </c>
-      <c r="Q4" s="25">
+      </c>
+      <c r="R4" s="25">
         <f t="shared" si="1"/>
-        <v>0.75</v>
-      </c>
-      <c r="R4" s="24">
+      </c>
+      <c r="S4" s="24">
         <f t="shared" si="2"/>
-        <v>3</v>
-      </c>
-      <c r="S4" s="2"/>
+      </c>
       <c r="T4" s="2"/>
       <c r="U4" s="2"/>
-    </row>
-    <row r="5" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V4" s="2"/>
+    </row>
+    <row r="5" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
       <c r="B5" s="2" t="s">
         <v>29</v>
@@ -7751,26 +7743,25 @@
         <v>1</v>
       </c>
       <c r="O5" s="24">
-        <f t="shared" ref="O5:O32" si="3">SUM(C5:N5)</f>
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="P5" s="24">
+        <f t="shared" ref="P5:P32" si="3">SUM(C5:O5)</f>
+      </c>
+      <c r="Q5" s="24">
         <f>VLOOKUP($B5,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>12</v>
-      </c>
-      <c r="Q5" s="25">
-        <f t="shared" ref="Q5:Q32" si="4">O5/P5</f>
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="R5" s="24">
-        <f t="shared" ref="R5:R32" si="5">P5-O5</f>
-        <v>4</v>
-      </c>
-      <c r="S5" s="2"/>
+      </c>
+      <c r="R5" s="25">
+        <f t="shared" ref="R5:R32" si="4">P5/Q5</f>
+      </c>
+      <c r="S5" s="24">
+        <f t="shared" ref="S5:S32" si="5">Q5-P5</f>
+      </c>
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
-    </row>
-    <row r="6" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V5" s="2"/>
+    </row>
+    <row r="6" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
         <v>30</v>
@@ -7812,26 +7803,25 @@
         <v>1</v>
       </c>
       <c r="O6" s="24">
+        <v>1</v>
+      </c>
+      <c r="P6" s="24">
         <f t="shared" si="3"/>
-        <v>8</v>
-      </c>
-      <c r="P6" s="24">
+      </c>
+      <c r="Q6" s="24">
         <f>VLOOKUP($B6,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>11</v>
-      </c>
-      <c r="Q6" s="25">
+      </c>
+      <c r="R6" s="25">
         <f t="shared" si="4"/>
-        <v>0.7272727272727273</v>
-      </c>
-      <c r="R6" s="24">
+      </c>
+      <c r="S6" s="24">
         <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="S6" s="2"/>
+      </c>
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
-    </row>
-    <row r="7" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V6" s="2"/>
+    </row>
+    <row r="7" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
         <v>39</v>
@@ -7873,26 +7863,25 @@
         <v>1</v>
       </c>
       <c r="O7" s="24">
+        <v>0</v>
+      </c>
+      <c r="P7" s="24">
         <f t="shared" si="3"/>
-        <v>7</v>
-      </c>
-      <c r="P7" s="24">
+      </c>
+      <c r="Q7" s="24">
         <f>VLOOKUP($B7,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>11</v>
-      </c>
-      <c r="Q7" s="25">
+      </c>
+      <c r="R7" s="25">
         <f t="shared" si="4"/>
-        <v>0.6363636363636364</v>
-      </c>
-      <c r="R7" s="24">
+      </c>
+      <c r="S7" s="24">
         <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
-      <c r="S7" s="2"/>
+      </c>
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
-    </row>
-    <row r="8" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V7" s="2"/>
+    </row>
+    <row r="8" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
       <c r="B8" s="2" t="s">
         <v>41</v>
@@ -7934,26 +7923,25 @@
         <v>0</v>
       </c>
       <c r="O8" s="24">
+        <v>1</v>
+      </c>
+      <c r="P8" s="24">
         <f t="shared" si="3"/>
-        <v>6</v>
-      </c>
-      <c r="P8" s="24">
+      </c>
+      <c r="Q8" s="24">
         <f>VLOOKUP($B8,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>10</v>
-      </c>
-      <c r="Q8" s="25">
+      </c>
+      <c r="R8" s="25">
         <f t="shared" si="4"/>
-        <v>0.6</v>
-      </c>
-      <c r="R8" s="24">
+      </c>
+      <c r="S8" s="24">
         <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
-      <c r="S8" s="2"/>
+      </c>
       <c r="T8" s="2"/>
       <c r="U8" s="2"/>
-    </row>
-    <row r="9" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V8" s="2"/>
+    </row>
+    <row r="9" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
       <c r="B9" s="2" t="s">
         <v>34</v>
@@ -7995,26 +7983,25 @@
         <v>18</v>
       </c>
       <c r="O9" s="24">
+        <v>0</v>
+      </c>
+      <c r="P9" s="24">
         <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="P9" s="24">
+      </c>
+      <c r="Q9" s="24">
         <f>VLOOKUP($B9,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>8</v>
-      </c>
-      <c r="Q9" s="25">
+      </c>
+      <c r="R9" s="25">
         <f t="shared" si="4"/>
-        <v>0.625</v>
-      </c>
-      <c r="R9" s="24">
+      </c>
+      <c r="S9" s="24">
         <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="S9" s="2"/>
+      </c>
       <c r="T9" s="2"/>
       <c r="U9" s="2"/>
-    </row>
-    <row r="10" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V9" s="2"/>
+    </row>
+    <row r="10" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
         <v>25</v>
@@ -8056,26 +8043,25 @@
         <v>1</v>
       </c>
       <c r="O10" s="24">
+        <v>1</v>
+      </c>
+      <c r="P10" s="24">
         <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="P10" s="24">
+      </c>
+      <c r="Q10" s="24">
         <f>VLOOKUP($B10,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>12</v>
-      </c>
-      <c r="Q10" s="25">
+      </c>
+      <c r="R10" s="25">
         <f t="shared" si="4"/>
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="R10" s="24">
+      </c>
+      <c r="S10" s="24">
         <f t="shared" si="5"/>
-        <v>7</v>
-      </c>
-      <c r="S10" s="2"/>
+      </c>
       <c r="T10" s="2"/>
       <c r="U10" s="2"/>
-    </row>
-    <row r="11" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V10" s="2"/>
+    </row>
+    <row r="11" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
       <c r="B11" s="2" t="s">
         <v>26</v>
@@ -8117,26 +8103,25 @@
         <v>1</v>
       </c>
       <c r="O11" s="24">
+        <v>0</v>
+      </c>
+      <c r="P11" s="24">
         <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="P11" s="24">
+      </c>
+      <c r="Q11" s="24">
         <f>VLOOKUP($B11,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>11</v>
-      </c>
-      <c r="Q11" s="25">
+      </c>
+      <c r="R11" s="25">
         <f t="shared" si="4"/>
-        <v>0.45454545454545453</v>
-      </c>
-      <c r="R11" s="24">
+      </c>
+      <c r="S11" s="24">
         <f t="shared" si="5"/>
-        <v>6</v>
-      </c>
-      <c r="S11" s="2"/>
+      </c>
       <c r="T11" s="2"/>
       <c r="U11" s="2"/>
-    </row>
-    <row r="12" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V11" s="2"/>
+    </row>
+    <row r="12" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
         <v>21</v>
@@ -8177,27 +8162,28 @@
       <c r="N12" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="O12" s="24">
+      <c r="O12" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P12" s="24">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="P12" s="24">
+      </c>
+      <c r="Q12" s="24">
         <f>VLOOKUP($B12,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>10</v>
-      </c>
-      <c r="Q12" s="25">
+      </c>
+      <c r="R12" s="25">
         <f t="shared" si="4"/>
-        <v>0.4</v>
-      </c>
-      <c r="R12" s="24">
+      </c>
+      <c r="S12" s="24">
         <f t="shared" si="5"/>
-        <v>6</v>
-      </c>
-      <c r="S12" s="2"/>
+      </c>
       <c r="T12" s="2"/>
       <c r="U12" s="2"/>
-    </row>
-    <row r="13" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V12" s="2"/>
+    </row>
+    <row r="13" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
       <c r="B13" s="2" t="s">
         <v>17</v>
@@ -8239,26 +8225,25 @@
         <v>18</v>
       </c>
       <c r="O13" s="24">
+        <v>1</v>
+      </c>
+      <c r="P13" s="24">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="P13" s="24">
+      </c>
+      <c r="Q13" s="24">
         <f>VLOOKUP($B13,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>10</v>
-      </c>
-      <c r="Q13" s="25">
+      </c>
+      <c r="R13" s="25">
         <f t="shared" si="4"/>
-        <v>0.4</v>
-      </c>
-      <c r="R13" s="24">
+      </c>
+      <c r="S13" s="24">
         <f t="shared" si="5"/>
-        <v>6</v>
-      </c>
-      <c r="S13" s="2"/>
+      </c>
       <c r="T13" s="2"/>
       <c r="U13" s="2"/>
-    </row>
-    <row r="14" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V13" s="2"/>
+    </row>
+    <row r="14" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
         <v>22</v>
@@ -8300,26 +8285,25 @@
         <v>0</v>
       </c>
       <c r="O14" s="24">
+        <v>1</v>
+      </c>
+      <c r="P14" s="24">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="P14" s="24">
+      </c>
+      <c r="Q14" s="24">
         <f>VLOOKUP($B14,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>6</v>
-      </c>
-      <c r="Q14" s="25">
+      </c>
+      <c r="R14" s="25">
         <f t="shared" si="4"/>
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="R14" s="24">
+      </c>
+      <c r="S14" s="24">
         <f t="shared" si="5"/>
-        <v>2</v>
-      </c>
-      <c r="S14" s="2"/>
+      </c>
       <c r="T14" s="2"/>
       <c r="U14" s="2"/>
-    </row>
-    <row r="15" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V14" s="2"/>
+    </row>
+    <row r="15" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
       <c r="B15" s="2" t="s">
         <v>28</v>
@@ -8361,26 +8345,25 @@
         <v>18</v>
       </c>
       <c r="O15" s="24">
+        <v>0</v>
+      </c>
+      <c r="P15" s="24">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="P15" s="24">
+      </c>
+      <c r="Q15" s="24">
         <f>VLOOKUP($B15,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>7</v>
-      </c>
-      <c r="Q15" s="25">
+      </c>
+      <c r="R15" s="25">
         <f t="shared" si="4"/>
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="R15" s="24">
+      </c>
+      <c r="S15" s="24">
         <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="S15" s="2"/>
+      </c>
       <c r="T15" s="2"/>
       <c r="U15" s="2"/>
-    </row>
-    <row r="16" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V15" s="2"/>
+    </row>
+    <row r="16" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
         <v>24</v>
@@ -8422,26 +8405,25 @@
         <v>0</v>
       </c>
       <c r="O16" s="24">
+        <v>0</v>
+      </c>
+      <c r="P16" s="24">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="P16" s="24">
+      </c>
+      <c r="Q16" s="24">
         <f>VLOOKUP($B16,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>12</v>
-      </c>
-      <c r="Q16" s="25">
+      </c>
+      <c r="R16" s="25">
         <f t="shared" si="4"/>
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="R16" s="24">
+      </c>
+      <c r="S16" s="24">
         <f t="shared" si="5"/>
-        <v>8</v>
-      </c>
-      <c r="S16" s="2"/>
+      </c>
       <c r="T16" s="2"/>
       <c r="U16" s="2"/>
-    </row>
-    <row r="17" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V16" s="2"/>
+    </row>
+    <row r="17" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
       <c r="B17" s="2" t="s">
         <v>36</v>
@@ -8483,26 +8465,25 @@
         <v>1</v>
       </c>
       <c r="O17" s="24">
+        <v>0</v>
+      </c>
+      <c r="P17" s="24">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="P17" s="24">
+      </c>
+      <c r="Q17" s="24">
         <f>VLOOKUP($B17,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>4</v>
-      </c>
-      <c r="Q17" s="25">
+      </c>
+      <c r="R17" s="25">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="R17" s="24">
+      </c>
+      <c r="S17" s="24">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="S17" s="2"/>
+      </c>
       <c r="T17" s="2"/>
       <c r="U17" s="2"/>
-    </row>
-    <row r="18" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V17" s="2"/>
+    </row>
+    <row r="18" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
       <c r="B18" s="2" t="s">
         <v>27</v>
@@ -8544,26 +8525,25 @@
         <v>1</v>
       </c>
       <c r="O18" s="24">
+        <v>1</v>
+      </c>
+      <c r="P18" s="24">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="P18" s="24">
+      </c>
+      <c r="Q18" s="24">
         <f>VLOOKUP($B18,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>11</v>
-      </c>
-      <c r="Q18" s="25">
+      </c>
+      <c r="R18" s="25">
         <f t="shared" si="4"/>
-        <v>0.36363636363636365</v>
-      </c>
-      <c r="R18" s="24">
+      </c>
+      <c r="S18" s="24">
         <f t="shared" si="5"/>
-        <v>7</v>
-      </c>
-      <c r="S18" s="2"/>
+      </c>
       <c r="T18" s="2"/>
       <c r="U18" s="2"/>
-    </row>
-    <row r="19" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V18" s="2"/>
+    </row>
+    <row r="19" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
       <c r="B19" s="2" t="s">
         <v>66</v>
@@ -8604,26 +8584,28 @@
       <c r="N19" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="O19" s="24">
+      <c r="O19" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P19" s="24">
         <f t="shared" si="3"/>
-        <v>3</v>
-      </c>
-      <c r="P19" s="24">
+      </c>
+      <c r="Q19" s="24">
         <v>6</v>
       </c>
-      <c r="Q19" s="25">
+      <c r="R19" s="25">
         <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-      <c r="R19" s="24">
+      </c>
+      <c r="S19" s="24">
         <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="S19" s="2"/>
+      </c>
       <c r="T19" s="2"/>
       <c r="U19" s="2"/>
-    </row>
-    <row r="20" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V19" s="2"/>
+    </row>
+    <row r="20" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
       <c r="B20" s="2" t="s">
         <v>31</v>
@@ -8665,26 +8647,25 @@
         <v>0</v>
       </c>
       <c r="O20" s="24">
+        <v>0</v>
+      </c>
+      <c r="P20" s="24">
         <f t="shared" si="3"/>
-        <v>3</v>
-      </c>
-      <c r="P20" s="24">
+      </c>
+      <c r="Q20" s="24">
         <f>VLOOKUP($B20,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>12</v>
-      </c>
-      <c r="Q20" s="25">
+      </c>
+      <c r="R20" s="25">
         <f t="shared" si="4"/>
-        <v>0.25</v>
-      </c>
-      <c r="R20" s="24">
+      </c>
+      <c r="S20" s="24">
         <f t="shared" si="5"/>
-        <v>9</v>
-      </c>
-      <c r="S20" s="2"/>
+      </c>
       <c r="T20" s="2"/>
       <c r="U20" s="2"/>
-    </row>
-    <row r="21" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V20" s="2"/>
+    </row>
+    <row r="21" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
       <c r="B21" s="2" t="s">
         <v>33</v>
@@ -8726,26 +8707,25 @@
         <v>1</v>
       </c>
       <c r="O21" s="24">
+        <v>0</v>
+      </c>
+      <c r="P21" s="24">
         <f t="shared" si="3"/>
-        <v>3</v>
-      </c>
-      <c r="P21" s="24">
+      </c>
+      <c r="Q21" s="24">
         <f>VLOOKUP($B21,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>11</v>
-      </c>
-      <c r="Q21" s="25">
+      </c>
+      <c r="R21" s="25">
         <f t="shared" si="4"/>
-        <v>0.2727272727272727</v>
-      </c>
-      <c r="R21" s="24">
+      </c>
+      <c r="S21" s="24">
         <f t="shared" si="5"/>
-        <v>8</v>
-      </c>
-      <c r="S21" s="2"/>
+      </c>
       <c r="T21" s="2"/>
       <c r="U21" s="2"/>
-    </row>
-    <row r="22" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V21" s="2"/>
+    </row>
+    <row r="22" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
       <c r="B22" s="2" t="s">
         <v>38</v>
@@ -8787,26 +8767,25 @@
         <v>1</v>
       </c>
       <c r="O22" s="24">
+        <v>1</v>
+      </c>
+      <c r="P22" s="24">
         <f t="shared" si="3"/>
-        <v>3</v>
-      </c>
-      <c r="P22" s="24">
+      </c>
+      <c r="Q22" s="24">
         <f>VLOOKUP($B22,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>7</v>
-      </c>
-      <c r="Q22" s="25">
+      </c>
+      <c r="R22" s="25">
         <f t="shared" si="4"/>
-        <v>0.42857142857142855</v>
-      </c>
-      <c r="R22" s="24">
+      </c>
+      <c r="S22" s="24">
         <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
-      <c r="S22" s="2"/>
+      </c>
       <c r="T22" s="2"/>
       <c r="U22" s="2"/>
-    </row>
-    <row r="23" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V22" s="2"/>
+    </row>
+    <row r="23" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
       <c r="B23" s="2" t="s">
         <v>67</v>
@@ -8847,26 +8826,28 @@
       <c r="N23" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="O23" s="24">
+      <c r="O23" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P23" s="24">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="P23" s="24">
+      </c>
+      <c r="Q23" s="24">
         <v>4</v>
       </c>
-      <c r="Q23" s="25">
+      <c r="R23" s="25">
         <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-      <c r="R23" s="24">
+      </c>
+      <c r="S23" s="24">
         <f t="shared" si="5"/>
-        <v>2</v>
-      </c>
-      <c r="S23" s="2"/>
+      </c>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
-    </row>
-    <row r="24" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V23" s="2"/>
+    </row>
+    <row r="24" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
       <c r="B24" s="2" t="s">
         <v>40</v>
@@ -8908,26 +8889,25 @@
         <v>18</v>
       </c>
       <c r="O24" s="24">
+        <v>0</v>
+      </c>
+      <c r="P24" s="24">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="P24" s="24">
+      </c>
+      <c r="Q24" s="24">
         <f>VLOOKUP($B24,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>8</v>
-      </c>
-      <c r="Q24" s="25">
+      </c>
+      <c r="R24" s="25">
         <f t="shared" si="4"/>
-        <v>0.25</v>
-      </c>
-      <c r="R24" s="24">
+      </c>
+      <c r="S24" s="24">
         <f t="shared" si="5"/>
-        <v>6</v>
-      </c>
-      <c r="S24" s="2"/>
+      </c>
       <c r="T24" s="2"/>
       <c r="U24" s="2"/>
-    </row>
-    <row r="25" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V24" s="2"/>
+    </row>
+    <row r="25" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
       <c r="B25" s="2" t="s">
         <v>23</v>
@@ -8969,26 +8949,25 @@
         <v>0</v>
       </c>
       <c r="O25" s="24">
+        <v>1</v>
+      </c>
+      <c r="P25" s="24">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="P25" s="24">
+      </c>
+      <c r="Q25" s="24">
         <f>VLOOKUP($B25,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>5</v>
-      </c>
-      <c r="Q25" s="25">
+      </c>
+      <c r="R25" s="25">
         <f t="shared" si="4"/>
-        <v>0.4</v>
-      </c>
-      <c r="R25" s="24">
+      </c>
+      <c r="S25" s="24">
         <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="S25" s="2"/>
+      </c>
       <c r="T25" s="2"/>
       <c r="U25" s="2"/>
-    </row>
-    <row r="26" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V25" s="2"/>
+    </row>
+    <row r="26" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
       <c r="B26" s="2" t="s">
         <v>35</v>
@@ -9030,26 +9009,25 @@
         <v>18</v>
       </c>
       <c r="O26" s="24">
+        <v>1</v>
+      </c>
+      <c r="P26" s="24">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="P26" s="24">
+      </c>
+      <c r="Q26" s="24">
         <f>VLOOKUP($B26,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>6</v>
-      </c>
-      <c r="Q26" s="25">
+      </c>
+      <c r="R26" s="25">
         <f t="shared" si="4"/>
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="R26" s="24">
+      </c>
+      <c r="S26" s="24">
         <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
-      <c r="S26" s="2"/>
+      </c>
       <c r="T26" s="2"/>
       <c r="U26" s="2"/>
-    </row>
-    <row r="27" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V26" s="2"/>
+    </row>
+    <row r="27" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
       <c r="B27" s="2" t="s">
         <v>63</v>
@@ -9091,26 +9069,25 @@
         <v>0</v>
       </c>
       <c r="O27" s="24">
+        <v>0</v>
+      </c>
+      <c r="P27" s="24">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="P27" s="24">
+      </c>
+      <c r="Q27" s="24">
         <f>VLOOKUP($B27,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>3</v>
-      </c>
-      <c r="Q27" s="25">
+      </c>
+      <c r="R27" s="25">
         <f t="shared" si="4"/>
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="R27" s="24">
+      </c>
+      <c r="S27" s="24">
         <f t="shared" si="5"/>
-        <v>2</v>
-      </c>
-      <c r="S27" s="2"/>
+      </c>
       <c r="T27" s="2"/>
       <c r="U27" s="2"/>
-    </row>
-    <row r="28" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V27" s="2"/>
+    </row>
+    <row r="28" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
       <c r="B28" s="2" t="s">
         <v>68</v>
@@ -9151,26 +9128,28 @@
       <c r="N28" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="O28" s="24">
+      <c r="O28" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P28" s="24">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="P28" s="24">
-        <v>1</v>
-      </c>
-      <c r="Q28" s="25">
+      </c>
+      <c r="Q28" s="24">
+        <v>1</v>
+      </c>
+      <c r="R28" s="25">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="R28" s="24">
+      </c>
+      <c r="S28" s="24">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="S28" s="2"/>
+      </c>
       <c r="T28" s="2"/>
       <c r="U28" s="2"/>
-    </row>
-    <row r="29" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V28" s="2"/>
+    </row>
+    <row r="29" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
       <c r="B29" s="2" t="s">
         <v>69</v>
@@ -9211,26 +9190,28 @@
       <c r="N29" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="O29" s="24">
+      <c r="O29" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P29" s="24">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="P29" s="24">
+      </c>
+      <c r="Q29" s="24">
         <v>3</v>
       </c>
-      <c r="Q29" s="25">
+      <c r="R29" s="25">
         <f t="shared" si="4"/>
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="R29" s="24">
+      </c>
+      <c r="S29" s="24">
         <f t="shared" si="5"/>
-        <v>2</v>
-      </c>
-      <c r="S29" s="2"/>
+      </c>
       <c r="T29" s="2"/>
       <c r="U29" s="2"/>
-    </row>
-    <row r="30" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V29" s="2"/>
+    </row>
+    <row r="30" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
       <c r="B30" s="2" t="s">
         <v>20</v>
@@ -9272,26 +9253,25 @@
         <v>0</v>
       </c>
       <c r="O30" s="24">
+        <v>1</v>
+      </c>
+      <c r="P30" s="24">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="P30" s="24">
+      </c>
+      <c r="Q30" s="24">
         <f>VLOOKUP($B30,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>2</v>
-      </c>
-      <c r="Q30" s="25">
+      </c>
+      <c r="R30" s="25">
         <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-      <c r="R30" s="24">
+      </c>
+      <c r="S30" s="24">
         <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-      <c r="S30" s="2"/>
+      </c>
       <c r="T30" s="2"/>
       <c r="U30" s="2"/>
-    </row>
-    <row r="31" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V30" s="2"/>
+    </row>
+    <row r="31" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
       <c r="B31" s="2" t="s">
         <v>70</v>
@@ -9332,26 +9312,28 @@
       <c r="N31" s="24">
         <v>1</v>
       </c>
-      <c r="O31" s="24">
+      <c r="O31" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P31" s="24">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="P31" s="24">
-        <v>1</v>
-      </c>
-      <c r="Q31" s="25">
+      </c>
+      <c r="Q31" s="24">
+        <v>1</v>
+      </c>
+      <c r="R31" s="25">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="R31" s="24">
+      </c>
+      <c r="S31" s="24">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="S31" s="2"/>
+      </c>
       <c r="T31" s="2"/>
       <c r="U31" s="2"/>
-    </row>
-    <row r="32" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V31" s="2"/>
+    </row>
+    <row r="32" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
       <c r="B32" s="2" t="s">
         <v>37</v>
@@ -9393,26 +9375,25 @@
         <v>0</v>
       </c>
       <c r="O32" s="24">
+        <v>0</v>
+      </c>
+      <c r="P32" s="24">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="P32" s="24">
+      </c>
+      <c r="Q32" s="24">
         <f>VLOOKUP($B32,Points!$B$2:$C$34,2,FALSE())</f>
-        <v>2</v>
-      </c>
-      <c r="Q32" s="25">
+      </c>
+      <c r="R32" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="R32" s="24">
+      </c>
+      <c r="S32" s="24">
         <f t="shared" si="5"/>
-        <v>2</v>
-      </c>
-      <c r="S32" s="2"/>
+      </c>
       <c r="T32" s="2"/>
       <c r="U32" s="2"/>
-    </row>
-    <row r="33" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V32" s="2"/>
+    </row>
+    <row r="33" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>
       <c r="B33" s="2" t="s">
         <v>72</v>
@@ -9453,17 +9434,22 @@
       <c r="N33" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="O33" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="P33" s="2"/>
+      <c r="O33" s="26" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P33" s="26" t="s">
+        <v>18</v>
+      </c>
       <c r="Q33" s="2"/>
       <c r="R33" s="2"/>
       <c r="S33" s="2"/>
       <c r="T33" s="2"/>
       <c r="U33" s="2"/>
-    </row>
-    <row r="34" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V33" s="2"/>
+    </row>
+    <row r="34" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
       <c r="B34" s="2" t="s">
         <v>48</v>
@@ -9518,19 +9504,20 @@
       </c>
       <c r="O34" s="24">
         <f>SUM(O3:O33)</f>
-        <v>116</v>
       </c>
       <c r="P34" s="24">
         <f>SUM(P3:P33)</f>
-        <v>230</v>
-      </c>
-      <c r="Q34" s="2"/>
+      </c>
+      <c r="Q34" s="24">
+        <f>SUM(Q3:Q33)</f>
+      </c>
       <c r="R34" s="2"/>
       <c r="S34" s="2"/>
       <c r="T34" s="2"/>
       <c r="U34" s="2"/>
-    </row>
-    <row r="35" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V34" s="2"/>
+    </row>
+    <row r="35" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -9552,8 +9539,9 @@
       <c r="S35" s="2"/>
       <c r="T35" s="2"/>
       <c r="U35" s="2"/>
-    </row>
-    <row r="36" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V35" s="2"/>
+    </row>
+    <row r="36" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -9575,8 +9563,9 @@
       <c r="S36" s="2"/>
       <c r="T36" s="2"/>
       <c r="U36" s="2"/>
-    </row>
-    <row r="37" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V36" s="2"/>
+    </row>
+    <row r="37" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -9598,8 +9587,9 @@
       <c r="S37" s="2"/>
       <c r="T37" s="2"/>
       <c r="U37" s="2"/>
-    </row>
-    <row r="38" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V37" s="2"/>
+    </row>
+    <row r="38" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -9621,8 +9611,9 @@
       <c r="S38" s="2"/>
       <c r="T38" s="2"/>
       <c r="U38" s="2"/>
-    </row>
-    <row r="39" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V38" s="2"/>
+    </row>
+    <row r="39" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -9644,8 +9635,9 @@
       <c r="S39" s="2"/>
       <c r="T39" s="2"/>
       <c r="U39" s="2"/>
-    </row>
-    <row r="40" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V39" s="2"/>
+    </row>
+    <row r="40" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="8"/>
       <c r="B40" s="8"/>
       <c r="C40" s="8"/>
@@ -9654,12 +9646,12 @@
       <c r="F40" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="B3:R31" xr:uid="{00000000-0009-0000-0000-000002000000}">
+  <autoFilter ref="B3:S31" xr:uid="{00000000-0009-0000-0000-000002000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:R31">
       <sortCondition descending="1" ref="C4:C31"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="C3:N32">
+  <conditionalFormatting sqref="C3:O32">
     <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
Fill DeOteris FBC 8-10 handicap indexes (12.8, 12.5, X)
Source: Handicaps_FBC_8_Final.xlsx and Handicaps_FBC_9_Final.xlsx; not in the
FBC 10 file (did not play). Sandbagger re-run with the new average.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vM3RZF9CPPLM8LSwSGoHo
</commit_message>
<xml_diff>
--- a/Handicaps & Points (Historical).xlsx
+++ b/Handicaps & Points (Historical).xlsx
@@ -1224,9 +1224,15 @@
       <c r="H9" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10"/>
+      <c r="I9" s="10">
+        <v>12.8</v>
+      </c>
+      <c r="J9" s="10">
+        <v>12.5</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>18</v>
+      </c>
       <c r="L9" s="10" t="s">
         <v>18</v>
       </c>
@@ -1239,23 +1245,18 @@
       <c r="O9" s="11"/>
       <c r="P9" s="10">
         <f>AVERAGE(C9:N9)</f>
-        <v>11.850000000000001</v>
       </c>
       <c r="Q9" s="10">
         <f>STDEV(C9:N9)</f>
-        <v>0.777817459305202</v>
       </c>
       <c r="R9" s="10">
         <f>MAX(C9:N9)</f>
-        <v>12.4</v>
       </c>
       <c r="S9" s="10">
         <f>MIN(C9:N9)</f>
-        <v>11.3</v>
       </c>
       <c r="T9" s="10">
         <f>R9-S9</f>
-        <v>1.0999999999999996</v>
       </c>
       <c r="U9" s="8"/>
     </row>

</xml_diff>

<commit_message>
Historical Cups: fix Fogan FBC 12 (0, lost) and Bussiculo FBC 11 (X, did not play)
Both now match FBC_Data, the By-Laws champions list and the live site.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vM3RZF9CPPLM8LSwSGoHo
</commit_message>
<xml_diff>
--- a/Handicaps & Points (Historical).xlsx
+++ b/Handicaps & Points (Historical).xlsx
@@ -8101,7 +8101,7 @@
         <v>1</v>
       </c>
       <c r="N11" s="24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O11" s="24">
         <v>0</v>
@@ -8579,8 +8579,8 @@
       <c r="L19" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="M19" s="24">
-        <v>0</v>
+      <c r="M19" s="24" t="s">
+        <v>18</v>
       </c>
       <c r="N19" s="24" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Cups: fix participation for Norat FBC 2, Bussiculo FBC 5 (did not play) and Weisberger FBC 4 (played, lost)
Each now matches the Archives match rows. Played counts updated; analytics
re-run (no table changed).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vM3RZF9CPPLM8LSwSGoHo
</commit_message>
<xml_diff>
--- a/Handicaps & Points (Historical).xlsx
+++ b/Handicaps & Points (Historical).xlsx
@@ -8561,8 +8561,8 @@
       <c r="F19" s="24">
         <v>1</v>
       </c>
-      <c r="G19" s="24">
-        <v>0</v>
+      <c r="G19" s="24" t="s">
+        <v>18</v>
       </c>
       <c r="H19" s="24">
         <v>1</v>
@@ -8594,7 +8594,7 @@
         <f t="shared" si="3"/>
       </c>
       <c r="Q19" s="24">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R19" s="25">
         <f t="shared" si="4"/>
@@ -8976,8 +8976,8 @@
       <c r="C26" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="D26" s="24">
-        <v>0</v>
+      <c r="D26" s="24" t="s">
+        <v>18</v>
       </c>
       <c r="E26" s="24">
         <v>0</v>
@@ -9164,8 +9164,8 @@
       <c r="E29" s="24">
         <v>1</v>
       </c>
-      <c r="F29" s="24" t="s">
-        <v>18</v>
+      <c r="F29" s="24">
+        <v>0</v>
       </c>
       <c r="G29" s="24" t="s">
         <v>18</v>

</xml_diff>